<commit_message>
add new field "Alias_BAUS" to better map corresponding runs for the affordable metrics
</commit_message>
<xml_diff>
--- a/utilities/RTP/config_RTP2025/ModelRuns_RTP2025.xlsx
+++ b/utilities/RTP/config_RTP2025/ModelRuns_RTP2025.xlsx
@@ -1,21 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ywang\Documents\GitHub\travel-model-one\utilities\RTP\config_RTP2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\travel-model-one\utilities\RTP\config_RTP2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28B37393-DD39-4478-A2C5-676558E892B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABA6695F-CAC3-4258-B7EB-7323CE9774B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="2304" windowWidth="25416" windowHeight="13284" xr2:uid="{1F9DB3D6-6479-4470-B3F5-B9ED0E0652FB}"/>
+    <workbookView xWindow="840" yWindow="6024" windowWidth="25416" windowHeight="11304" xr2:uid="{1F9DB3D6-6479-4470-B3F5-B9ED0E0652FB}"/>
   </bookViews>
   <sheets>
     <sheet name="ModelRuns" sheetId="1" r:id="rId1"/>
     <sheet name="Estimating Constants" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ModelRuns!$A$1:$Z$298</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -77,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3488" uniqueCount="1129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3500" uniqueCount="1130">
   <si>
     <t>year</t>
   </si>
@@ -3464,6 +3467,9 @@
   </si>
   <si>
     <t>2050 FBP minus T12</t>
+  </si>
+  <si>
+    <t>Alias_BAUS</t>
   </si>
 </sst>
 </file>
@@ -3475,7 +3481,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3587,6 +3593,13 @@
       <i/>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -3899,7 +3912,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="257">
+  <cellXfs count="258">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4339,6 +4352,9 @@
     <xf numFmtId="0" fontId="2" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4669,7 +4685,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9564CC59-3725-4FDA-8BF2-0F68CB1B6F5A}">
-  <dimension ref="A1:Y298"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:Z298"/>
   <sheetFormatPr defaultColWidth="9.33203125" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" style="1" bestFit="1" customWidth="1"/>
@@ -4687,10 +4704,13 @@
     <col min="13" max="13" width="17.5546875" style="1" customWidth="1"/>
     <col min="14" max="14" width="8.33203125" style="1" customWidth="1"/>
     <col min="15" max="16" width="9.33203125" style="41"/>
-    <col min="17" max="16384" width="9.33203125" style="1"/>
+    <col min="17" max="24" width="9.33203125" style="1"/>
+    <col min="25" max="25" width="14.33203125" style="1" customWidth="1"/>
+    <col min="26" max="26" width="13.44140625" style="1" customWidth="1"/>
+    <col min="27" max="16384" width="9.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" s="5" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" s="5" customFormat="1" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -4766,8 +4786,11 @@
       <c r="Y1" s="2" t="s">
         <v>329</v>
       </c>
-    </row>
-    <row r="2" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="Z1" s="257" t="s">
+        <v>1129</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" s="20" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="18">
         <v>2005</v>
       </c>
@@ -4823,7 +4846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:25" s="29" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="28">
         <v>2005</v>
       </c>
@@ -4882,7 +4905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:25" s="29" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="28">
         <v>2005</v>
       </c>
@@ -4937,7 +4960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:25" s="29" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26" s="29" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="28">
         <v>2005</v>
       </c>
@@ -4992,7 +5015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:25" s="29" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26" s="29" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="28">
         <v>2005</v>
       </c>
@@ -5056,8 +5079,11 @@
       <c r="X6" s="31">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:25" s="126" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="Z6" s="29">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" s="126" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="125">
         <v>2005</v>
       </c>
@@ -5124,8 +5150,11 @@
       <c r="Y7" s="130" t="s">
         <v>415</v>
       </c>
-    </row>
-    <row r="8" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="Z7" s="126">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" s="51" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="50">
         <v>2015</v>
       </c>
@@ -5169,7 +5198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:25" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" s="33" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="32">
         <v>2015</v>
       </c>
@@ -5218,7 +5247,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:25" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" s="33" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="32">
         <v>2015</v>
       </c>
@@ -5274,7 +5303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:25" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" s="33" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="32">
         <v>2015</v>
       </c>
@@ -5330,7 +5359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:25" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" s="33" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="32">
         <v>2015</v>
       </c>
@@ -5386,7 +5415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:25" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" s="33" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="32">
         <v>2015</v>
       </c>
@@ -5445,7 +5474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:25" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:26" s="33" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="32">
         <v>2015</v>
       </c>
@@ -5504,7 +5533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:25" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:26" s="33" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="32">
         <v>2015</v>
       </c>
@@ -5563,7 +5592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:25" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:26" s="33" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="32">
         <v>2015</v>
       </c>
@@ -5623,7 +5652,7 @@
       </c>
       <c r="Y16" s="55"/>
     </row>
-    <row r="17" spans="1:25" s="33" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:26" s="33" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="32">
         <v>2015</v>
       </c>
@@ -5689,8 +5718,11 @@
       <c r="Y17" s="55" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="18" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="Z17" s="33">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26" s="51" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="51">
         <v>2015</v>
       </c>
@@ -5749,7 +5781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:26" s="51" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="51">
         <v>2015</v>
       </c>
@@ -5808,7 +5840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:26" s="51" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="51">
         <v>2015</v>
       </c>
@@ -5867,7 +5899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:26" s="51" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="51">
         <v>2015</v>
       </c>
@@ -5926,7 +5958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:26" s="51" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="51">
         <v>2015</v>
       </c>
@@ -5987,7 +6019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:26" s="51" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="51">
         <v>2015</v>
       </c>
@@ -6048,7 +6080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:26" s="51" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="51">
         <v>2015</v>
       </c>
@@ -6107,7 +6139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:26" s="51" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="51">
         <v>2015</v>
       </c>
@@ -6166,7 +6198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:26" s="51" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="51">
         <v>2015</v>
       </c>
@@ -6226,7 +6258,7 @@
       </c>
       <c r="Y26" s="132"/>
     </row>
-    <row r="27" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:26" s="51" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="51">
         <v>2015</v>
       </c>
@@ -6290,8 +6322,11 @@
       <c r="Y27" s="132" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z27" s="51">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="28" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>2023</v>
       </c>
@@ -6340,7 +6375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>2023</v>
       </c>
@@ -6389,7 +6424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>2023</v>
       </c>
@@ -6438,7 +6473,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>2023</v>
       </c>
@@ -6487,7 +6522,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:26" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>2023</v>
       </c>
@@ -6536,7 +6571,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="33" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>2023</v>
       </c>
@@ -6585,7 +6620,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>2023</v>
       </c>
@@ -6634,7 +6669,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>2023</v>
       </c>
@@ -6683,7 +6718,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>2023</v>
       </c>
@@ -6732,7 +6767,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>2023</v>
       </c>
@@ -6781,7 +6816,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="38" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>2023</v>
       </c>
@@ -6830,7 +6865,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>2023</v>
       </c>
@@ -6879,7 +6914,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>2023</v>
       </c>
@@ -6928,7 +6963,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>2023</v>
       </c>
@@ -6977,7 +7012,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>2023</v>
       </c>
@@ -7026,7 +7061,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>2023</v>
       </c>
@@ -7075,7 +7110,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
         <v>2023</v>
       </c>
@@ -7124,7 +7159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
         <v>2023</v>
       </c>
@@ -7173,7 +7208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
         <v>2023</v>
       </c>
@@ -7220,7 +7255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
         <v>2023</v>
       </c>
@@ -7272,7 +7307,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="48" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
         <v>2023</v>
       </c>
@@ -7322,7 +7357,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="49" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
         <v>2023</v>
       </c>
@@ -7374,7 +7409,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="50" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1">
         <v>2023</v>
       </c>
@@ -7433,7 +7468,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="51" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1">
         <v>2023</v>
       </c>
@@ -7492,7 +7527,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="52" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1">
         <v>2023</v>
       </c>
@@ -7551,7 +7586,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="53" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1">
         <v>2023</v>
       </c>
@@ -7610,7 +7645,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="54" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1">
         <v>2023</v>
       </c>
@@ -7669,7 +7704,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="55" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1">
         <v>2023</v>
       </c>
@@ -7728,7 +7763,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="56" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1">
         <v>2023</v>
       </c>
@@ -7787,7 +7822,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="57" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1">
         <v>2023</v>
       </c>
@@ -7846,7 +7881,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="58" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1">
         <v>2023</v>
       </c>
@@ -7905,7 +7940,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="59" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1">
         <v>2023</v>
       </c>
@@ -7964,7 +7999,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="60" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1">
         <v>2023</v>
       </c>
@@ -8023,7 +8058,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="61" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1">
         <v>2023</v>
       </c>
@@ -8082,7 +8117,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="62" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1">
         <v>2023</v>
       </c>
@@ -8141,7 +8176,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="63" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1">
         <v>2023</v>
       </c>
@@ -8200,7 +8235,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="64" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1">
         <v>2023</v>
       </c>
@@ -8259,7 +8294,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="65" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1">
         <v>2023</v>
       </c>
@@ -8318,7 +8353,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="66" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1">
         <v>2023</v>
       </c>
@@ -8377,7 +8412,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="67" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1">
         <v>2023</v>
       </c>
@@ -8436,7 +8471,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="68" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1">
         <v>2023</v>
       </c>
@@ -8495,7 +8530,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="69" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1">
         <v>2023</v>
       </c>
@@ -8554,7 +8589,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="70" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1">
         <v>2023</v>
       </c>
@@ -8613,7 +8648,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="71" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="1">
         <v>2023</v>
       </c>
@@ -8672,7 +8707,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="72" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="1">
         <v>2023</v>
       </c>
@@ -8731,7 +8766,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="73" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1">
         <v>2023</v>
       </c>
@@ -8790,7 +8825,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="74" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1">
         <v>2023</v>
       </c>
@@ -8849,7 +8884,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="75" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1">
         <v>2023</v>
       </c>
@@ -8911,7 +8946,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="76" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1">
         <v>2023</v>
       </c>
@@ -8970,7 +9005,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1">
         <v>2023</v>
       </c>
@@ -9032,7 +9067,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="78" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1">
         <v>2023</v>
       </c>
@@ -9094,7 +9129,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="79" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1">
         <v>2023</v>
       </c>
@@ -9156,7 +9191,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="80" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1">
         <v>2023</v>
       </c>
@@ -9218,7 +9253,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="81" spans="1:24" ht="12.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:24" ht="12.45" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1">
         <v>2023</v>
       </c>
@@ -9277,7 +9312,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="82" spans="1:24" ht="12.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:24" ht="12.45" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1">
         <v>2023</v>
       </c>
@@ -9336,7 +9371,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="83" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="1">
         <v>2023</v>
       </c>
@@ -9395,7 +9430,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="84" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="1">
         <v>2023</v>
       </c>
@@ -9454,7 +9489,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="85" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" s="1">
         <v>2023</v>
       </c>
@@ -9513,7 +9548,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="86" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" s="1">
         <v>2023</v>
       </c>
@@ -9572,7 +9607,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="87" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" s="1">
         <v>2023</v>
       </c>
@@ -9631,7 +9666,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="88" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" s="1">
         <v>2023</v>
       </c>
@@ -9690,7 +9725,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="89" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" s="93">
         <v>2023</v>
       </c>
@@ -9749,7 +9784,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="90" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" s="93">
         <v>2023</v>
       </c>
@@ -9808,7 +9843,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="91" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" s="93">
         <v>2023</v>
       </c>
@@ -9867,7 +9902,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="92" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" s="93">
         <v>2023</v>
       </c>
@@ -9926,7 +9961,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="93" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="93">
         <v>2023</v>
       </c>
@@ -9985,7 +10020,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="94" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" s="93">
         <v>2023</v>
       </c>
@@ -10044,7 +10079,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="95" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" s="93">
         <v>2023</v>
       </c>
@@ -10103,7 +10138,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="96" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" s="93">
         <v>2023</v>
       </c>
@@ -10162,7 +10197,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="97" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" s="93">
         <v>2023</v>
       </c>
@@ -10223,7 +10258,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="98" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" s="93">
         <v>2023</v>
       </c>
@@ -10280,7 +10315,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="99" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" s="93">
         <v>2023</v>
       </c>
@@ -10337,7 +10372,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="100" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="93">
         <v>2023</v>
       </c>
@@ -10394,7 +10429,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="101" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="93">
         <v>2023</v>
       </c>
@@ -10451,7 +10486,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="102" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="93">
         <v>2023</v>
       </c>
@@ -10508,7 +10543,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="103" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="93">
         <v>2023</v>
       </c>
@@ -10565,7 +10600,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="104" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" s="93">
         <v>2023</v>
       </c>
@@ -10622,7 +10657,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="105" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="93">
         <v>2023</v>
       </c>
@@ -10679,7 +10714,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="106" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" s="93">
         <v>2023</v>
       </c>
@@ -10736,7 +10771,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="107" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="93">
         <v>2023</v>
       </c>
@@ -10793,7 +10828,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="108" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="93">
         <v>2023</v>
       </c>
@@ -10852,7 +10887,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="109" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="93">
         <v>2023</v>
       </c>
@@ -10911,7 +10946,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="110" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" s="93">
         <v>2023</v>
       </c>
@@ -10970,7 +11005,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="111" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="93">
         <v>2023</v>
       </c>
@@ -11029,7 +11064,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="112" spans="1:24" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:24" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" s="93">
         <v>2023</v>
       </c>
@@ -11088,7 +11123,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="113" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="93">
         <v>2023</v>
       </c>
@@ -11147,7 +11182,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="114" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" s="93">
         <v>2023</v>
       </c>
@@ -11206,7 +11241,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="115" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" s="93">
         <v>2023</v>
       </c>
@@ -11265,7 +11300,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="116" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" s="93">
         <v>2023</v>
       </c>
@@ -11324,7 +11359,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="117" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="93">
         <v>2023</v>
       </c>
@@ -11383,7 +11418,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="118" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="93">
         <v>2023</v>
       </c>
@@ -11442,7 +11477,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="119" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="93">
         <v>2023</v>
       </c>
@@ -11501,7 +11536,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="120" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" s="93">
         <v>2023</v>
       </c>
@@ -11561,7 +11596,7 @@
       </c>
       <c r="Y120" s="133"/>
     </row>
-    <row r="121" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" s="93">
         <v>2023</v>
       </c>
@@ -11621,7 +11656,7 @@
       </c>
       <c r="Y121" s="133"/>
     </row>
-    <row r="122" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" s="93">
         <v>2023</v>
       </c>
@@ -11681,7 +11716,7 @@
       </c>
       <c r="Y122" s="133"/>
     </row>
-    <row r="123" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="93">
         <v>2023</v>
       </c>
@@ -11741,7 +11776,7 @@
       </c>
       <c r="Y123" s="133"/>
     </row>
-    <row r="124" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" s="93">
         <v>2023</v>
       </c>
@@ -11800,7 +11835,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="125" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:26" s="93" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A125" s="93">
         <v>2023</v>
       </c>
@@ -11864,8 +11899,11 @@
       <c r="Y125" s="133" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="126" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="Z125" s="93">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="126" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" s="93">
         <v>2023</v>
       </c>
@@ -11925,7 +11963,7 @@
       </c>
       <c r="Y126" s="133"/>
     </row>
-    <row r="127" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" s="93">
         <v>2023</v>
       </c>
@@ -11985,7 +12023,7 @@
       </c>
       <c r="Y127" s="133"/>
     </row>
-    <row r="128" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" s="93">
         <v>2023</v>
       </c>
@@ -12045,7 +12083,7 @@
       </c>
       <c r="Y128" s="133"/>
     </row>
-    <row r="129" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:25" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="93">
         <v>2023</v>
       </c>
@@ -12105,7 +12143,7 @@
       </c>
       <c r="Y129" s="133"/>
     </row>
-    <row r="130" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:25" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="93">
         <v>2023</v>
       </c>
@@ -12165,7 +12203,7 @@
       </c>
       <c r="Y130" s="133"/>
     </row>
-    <row r="131" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:25" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="93">
         <v>2023</v>
       </c>
@@ -12225,7 +12263,7 @@
       </c>
       <c r="Y131" s="133"/>
     </row>
-    <row r="132" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:25" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" s="93">
         <v>2023</v>
       </c>
@@ -12285,7 +12323,7 @@
       </c>
       <c r="Y132" s="133"/>
     </row>
-    <row r="133" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:25" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" s="93">
         <v>2023</v>
       </c>
@@ -12353,7 +12391,7 @@
         <v>967</v>
       </c>
     </row>
-    <row r="134" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:25" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" s="93">
         <v>2023</v>
       </c>
@@ -12421,7 +12459,7 @@
         <v>968</v>
       </c>
     </row>
-    <row r="135" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:25" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" s="93">
         <v>2023</v>
       </c>
@@ -12489,7 +12527,7 @@
         <v>967</v>
       </c>
     </row>
-    <row r="136" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:25" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" s="93">
         <v>2023</v>
       </c>
@@ -12557,7 +12595,7 @@
         <v>968</v>
       </c>
     </row>
-    <row r="137" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:25" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" s="93">
         <v>2023</v>
       </c>
@@ -12625,7 +12663,7 @@
         <v>970</v>
       </c>
     </row>
-    <row r="138" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:25" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" s="93">
         <v>2023</v>
       </c>
@@ -12693,7 +12731,7 @@
         <v>969</v>
       </c>
     </row>
-    <row r="139" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:25" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" s="93">
         <v>2023</v>
       </c>
@@ -12761,7 +12799,7 @@
         <v>970</v>
       </c>
     </row>
-    <row r="140" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:25" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" s="93">
         <v>2023</v>
       </c>
@@ -12829,7 +12867,7 @@
         <v>970</v>
       </c>
     </row>
-    <row r="141" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:25" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" s="93">
         <v>2023</v>
       </c>
@@ -12897,7 +12935,7 @@
         <v>970</v>
       </c>
     </row>
-    <row r="142" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:25" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" s="93">
         <v>2023</v>
       </c>
@@ -12965,7 +13003,7 @@
         <v>982</v>
       </c>
     </row>
-    <row r="143" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:25" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" s="93">
         <v>2023</v>
       </c>
@@ -13033,7 +13071,7 @@
         <v>983</v>
       </c>
     </row>
-    <row r="144" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:25" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" s="93">
         <v>2023</v>
       </c>
@@ -13101,7 +13139,7 @@
         <v>984</v>
       </c>
     </row>
-    <row r="145" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" s="93">
         <v>2023</v>
       </c>
@@ -13169,7 +13207,7 @@
         <v>985</v>
       </c>
     </row>
-    <row r="146" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" s="93">
         <v>2023</v>
       </c>
@@ -13237,7 +13275,7 @@
         <v>1115</v>
       </c>
     </row>
-    <row r="147" spans="1:25" s="93" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:26" s="93" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" s="93">
         <v>2023</v>
       </c>
@@ -13305,7 +13343,7 @@
         <v>1116</v>
       </c>
     </row>
-    <row r="148" spans="1:25" s="107" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:26" s="107" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" s="107">
         <v>2025</v>
       </c>
@@ -13333,7 +13371,7 @@
       <c r="W148" s="111"/>
       <c r="X148" s="111"/>
     </row>
-    <row r="149" spans="1:25" s="25" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:26" s="25" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" s="25">
         <v>2025</v>
       </c>
@@ -13361,7 +13399,7 @@
       <c r="W149" s="27"/>
       <c r="X149" s="27"/>
     </row>
-    <row r="150" spans="1:25" s="107" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:26" s="107" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" s="107">
         <v>2030</v>
       </c>
@@ -13384,7 +13422,7 @@
       <c r="W150" s="111"/>
       <c r="X150" s="111"/>
     </row>
-    <row r="151" spans="1:25" s="25" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:26" s="25" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" s="25">
         <v>2030</v>
       </c>
@@ -13407,7 +13445,7 @@
       <c r="W151" s="27"/>
       <c r="X151" s="27"/>
     </row>
-    <row r="152" spans="1:25" s="176" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:26" s="176" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A152" s="176">
         <v>2030</v>
       </c>
@@ -13471,8 +13509,11 @@
       <c r="Y152" s="176" t="s">
         <v>909</v>
       </c>
-    </row>
-    <row r="153" spans="1:25" s="73" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="Z152" s="176" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="153" spans="1:26" s="73" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" s="73">
         <v>2035</v>
       </c>
@@ -13531,7 +13572,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="154" spans="1:25" s="15" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:26" s="15" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" s="15">
         <v>2035</v>
       </c>
@@ -13590,7 +13631,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="155" spans="1:25" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:26" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" s="12">
         <v>2035</v>
       </c>
@@ -13649,7 +13690,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="156" spans="1:25" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:26" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" s="12">
         <v>2035</v>
       </c>
@@ -13708,7 +13749,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="157" spans="1:25" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:26" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" s="12">
         <v>2035</v>
       </c>
@@ -13767,7 +13808,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:25" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:26" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" s="12">
         <v>2035</v>
       </c>
@@ -13823,7 +13864,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="159" spans="1:25" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:26" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" s="12">
         <v>2035</v>
       </c>
@@ -13879,7 +13920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:25" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:26" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" s="12">
         <v>2035</v>
       </c>
@@ -13935,7 +13976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:24" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" s="12">
         <v>2035</v>
       </c>
@@ -13991,7 +14032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:24" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" s="12">
         <v>2035</v>
       </c>
@@ -14047,7 +14088,7 @@
         <v>41.25</v>
       </c>
     </row>
-    <row r="163" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:24" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" s="12">
         <v>2035</v>
       </c>
@@ -14103,7 +14144,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="164" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:24" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" s="12">
         <v>2035</v>
       </c>
@@ -14159,7 +14200,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="165" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:24" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" s="12">
         <v>2035</v>
       </c>
@@ -14215,7 +14256,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="166" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:24" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" s="12">
         <v>2035</v>
       </c>
@@ -14271,7 +14312,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="167" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:24" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" s="12">
         <v>2035</v>
       </c>
@@ -14327,7 +14368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:24" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" s="12">
         <v>2035</v>
       </c>
@@ -14383,7 +14424,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="169" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:24" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" s="12">
         <v>2035</v>
       </c>
@@ -14439,7 +14480,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="170" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:24" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" s="12">
         <v>2035</v>
       </c>
@@ -14495,7 +14536,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="171" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:24" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" s="12">
         <v>2035</v>
       </c>
@@ -14554,7 +14595,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="172" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:24" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" s="12">
         <v>2035</v>
       </c>
@@ -14610,7 +14651,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="173" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:24" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" s="12">
         <v>2035</v>
       </c>
@@ -14666,7 +14707,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="174" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:24" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" s="12">
         <v>2035</v>
       </c>
@@ -14722,7 +14763,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="175" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:24" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" s="12">
         <v>2035</v>
       </c>
@@ -14778,7 +14819,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="176" spans="1:24" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:24" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" s="12">
         <v>2035</v>
       </c>
@@ -14896,7 +14937,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="178" spans="1:25" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:25" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" s="12">
         <v>2035</v>
       </c>
@@ -14952,7 +14993,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="179" spans="1:25" s="12" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:25" s="12" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" s="12">
         <v>2035</v>
       </c>
@@ -15076,7 +15117,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="181" spans="1:25" s="56" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:25" s="56" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" s="56">
         <v>2035</v>
       </c>
@@ -15132,7 +15173,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="182" spans="1:25" s="56" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:25" s="56" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" s="56">
         <v>2035</v>
       </c>
@@ -15188,7 +15229,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="183" spans="1:25" s="56" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:25" s="56" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" s="56">
         <v>2035</v>
       </c>
@@ -15244,7 +15285,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="184" spans="1:25" s="56" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:25" s="56" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" s="56">
         <v>2035</v>
       </c>
@@ -15303,7 +15344,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="185" spans="1:25" s="56" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:25" s="56" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" s="56">
         <v>2035</v>
       </c>
@@ -15362,7 +15403,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="186" spans="1:25" s="56" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:25" s="56" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" s="56">
         <v>2035</v>
       </c>
@@ -15483,7 +15524,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="188" spans="1:25" s="117" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:25" s="117" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" s="117">
         <v>2035</v>
       </c>
@@ -15539,7 +15580,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="189" spans="1:25" s="117" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:25" s="117" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" s="117">
         <v>2035</v>
       </c>
@@ -15595,7 +15636,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="190" spans="1:25" s="117" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:25" s="117" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" s="117">
         <v>2035</v>
       </c>
@@ -15651,7 +15692,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="191" spans="1:25" s="117" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:25" s="117" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" s="117">
         <v>2035</v>
       </c>
@@ -15707,7 +15748,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="192" spans="1:25" s="117" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:25" s="117" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" s="117">
         <v>2035</v>
       </c>
@@ -15763,7 +15804,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="193" spans="1:25" s="117" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:26" s="117" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A193" s="117">
         <v>2035</v>
       </c>
@@ -15825,7 +15866,7 @@
         <v>860</v>
       </c>
     </row>
-    <row r="194" spans="1:25" s="117" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:26" s="117" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194" s="117">
         <v>2035</v>
       </c>
@@ -15881,7 +15922,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="195" spans="1:25" s="117" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:26" s="117" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" s="117">
         <v>2035</v>
       </c>
@@ -15937,7 +15978,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="196" spans="1:25" s="117" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:26" s="117" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" s="117">
         <v>2035</v>
       </c>
@@ -15993,7 +16034,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="197" spans="1:25" s="117" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:26" s="117" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A197" s="117">
         <v>2035</v>
       </c>
@@ -16054,8 +16095,11 @@
       <c r="Y197" s="117" t="s">
         <v>694</v>
       </c>
-    </row>
-    <row r="198" spans="1:25" s="81" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="Z197" s="117" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="198" spans="1:26" s="81" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198" s="81">
         <v>2035</v>
       </c>
@@ -16111,7 +16155,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="199" spans="1:25" s="81" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:26" s="81" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" s="81">
         <v>2035</v>
       </c>
@@ -16170,7 +16214,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="200" spans="1:25" s="60" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:26" s="60" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" s="60">
         <v>2035</v>
       </c>
@@ -16226,7 +16270,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="201" spans="1:25" s="60" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:26" s="60" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" s="60">
         <v>2035</v>
       </c>
@@ -16282,7 +16326,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="202" spans="1:25" s="60" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:26" s="60" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" s="60">
         <v>2035</v>
       </c>
@@ -16338,7 +16382,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="203" spans="1:25" s="60" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:26" s="60" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" s="60">
         <v>2035</v>
       </c>
@@ -16397,7 +16441,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="204" spans="1:25" s="60" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:26" s="60" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" s="60">
         <v>2035</v>
       </c>
@@ -16456,7 +16500,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="205" spans="1:25" s="60" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:26" s="60" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" s="60">
         <v>2035</v>
       </c>
@@ -16515,7 +16559,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="206" spans="1:25" s="60" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:26" s="60" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206" s="60">
         <v>2035</v>
       </c>
@@ -16574,7 +16618,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="207" spans="1:25" s="60" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:26" s="60" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" s="60">
         <v>2035</v>
       </c>
@@ -16633,7 +16677,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="208" spans="1:25" s="60" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:26" s="60" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A208" s="60">
         <v>2035</v>
       </c>
@@ -16698,7 +16742,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="209" spans="1:25" s="117" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:26" s="117" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A209" s="117">
         <v>2035</v>
       </c>
@@ -16763,7 +16807,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="210" spans="1:25" s="60" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:26" s="60" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" s="60">
         <v>2035</v>
       </c>
@@ -16816,7 +16860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:25" s="60" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:26" s="60" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" s="60">
         <v>2035</v>
       </c>
@@ -16869,7 +16913,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="212" spans="1:25" s="60" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:26" s="60" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A212" s="60">
         <v>2035</v>
       </c>
@@ -16925,7 +16969,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="213" spans="1:25" s="117" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:26" s="117" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" s="117">
         <v>2035</v>
       </c>
@@ -16981,7 +17025,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="214" spans="1:25" s="117" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:26" s="117" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" s="117">
         <v>2035</v>
       </c>
@@ -17037,7 +17081,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="215" spans="1:25" s="117" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:26" s="117" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" s="117">
         <v>2035</v>
       </c>
@@ -17093,7 +17137,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="216" spans="1:25" s="117" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:26" s="117" customFormat="1" ht="14.4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216" s="117">
         <v>2035</v>
       </c>
@@ -17149,7 +17193,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="217" spans="1:25" s="117" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:26" s="117" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217" s="117">
         <v>2035</v>
       </c>
@@ -17205,7 +17249,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="218" spans="1:25" s="117" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:26" s="117" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218" s="117">
         <v>2035</v>
       </c>
@@ -17261,7 +17305,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="219" spans="1:25" s="117" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:26" s="117" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219" s="117">
         <v>2035</v>
       </c>
@@ -17317,7 +17361,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="220" spans="1:25" s="117" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:26" s="117" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A220" s="117">
         <v>2035</v>
       </c>
@@ -17373,7 +17417,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="221" spans="1:25" s="117" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:26" s="117" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221" s="117">
         <v>2035</v>
       </c>
@@ -17429,7 +17473,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="222" spans="1:25" s="117" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:26" s="117" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222" s="117">
         <v>2035</v>
       </c>
@@ -17485,7 +17529,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="223" spans="1:25" s="117" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:26" s="117" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223" s="117">
         <v>2035</v>
       </c>
@@ -17544,7 +17588,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="224" spans="1:25" s="117" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:26" s="117" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A224" s="117">
         <v>2035</v>
       </c>
@@ -17608,8 +17652,11 @@
       <c r="Y224" s="117" t="s">
         <v>358</v>
       </c>
-    </row>
-    <row r="225" spans="1:25" s="81" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="Z224" s="117" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="225" spans="1:26" s="81" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225" s="81">
         <v>2035</v>
       </c>
@@ -17668,7 +17715,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="226" spans="1:25" s="81" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:26" s="81" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A226" s="81">
         <v>2035</v>
       </c>
@@ -17732,8 +17779,11 @@
       <c r="Y226" s="81" t="s">
         <v>881</v>
       </c>
-    </row>
-    <row r="227" spans="1:25" s="162" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="Z226" s="81" t="s">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="227" spans="1:26" s="162" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A227" s="162">
         <v>2035</v>
       </c>
@@ -17797,8 +17847,11 @@
       <c r="Y227" s="162" t="s">
         <v>895</v>
       </c>
-    </row>
-    <row r="228" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="Z227" s="162" t="s">
+        <v>895</v>
+      </c>
+    </row>
+    <row r="228" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228" s="236">
         <v>2035</v>
       </c>
@@ -17863,7 +17916,7 @@
         <v>1066</v>
       </c>
     </row>
-    <row r="229" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229" s="236">
         <v>2035</v>
       </c>
@@ -17928,7 +17981,7 @@
         <v>1059</v>
       </c>
     </row>
-    <row r="230" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A230" s="236">
         <v>2035</v>
       </c>
@@ -17993,7 +18046,7 @@
         <v>999</v>
       </c>
     </row>
-    <row r="231" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231" s="236">
         <v>2035</v>
       </c>
@@ -18058,7 +18111,7 @@
         <v>1001</v>
       </c>
     </row>
-    <row r="232" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A232" s="236">
         <v>2035</v>
       </c>
@@ -18123,7 +18176,7 @@
         <v>1010</v>
       </c>
     </row>
-    <row r="233" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A233" s="236">
         <v>2035</v>
       </c>
@@ -18188,7 +18241,7 @@
         <v>1011</v>
       </c>
     </row>
-    <row r="234" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A234" s="236">
         <v>2035</v>
       </c>
@@ -18253,7 +18306,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="235" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A235" s="236">
         <v>2035</v>
       </c>
@@ -18318,7 +18371,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="236" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A236" s="236">
         <v>2035</v>
       </c>
@@ -18383,7 +18436,7 @@
         <v>1067</v>
       </c>
     </row>
-    <row r="237" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A237" s="236">
         <v>2035</v>
       </c>
@@ -18448,7 +18501,7 @@
         <v>1068</v>
       </c>
     </row>
-    <row r="238" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238" s="236">
         <v>2035</v>
       </c>
@@ -18513,7 +18566,7 @@
         <v>1069</v>
       </c>
     </row>
-    <row r="239" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A239" s="236">
         <v>2035</v>
       </c>
@@ -18578,7 +18631,7 @@
         <v>1070</v>
       </c>
     </row>
-    <row r="240" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A240" s="236">
         <v>2035</v>
       </c>
@@ -18643,7 +18696,7 @@
         <v>1071</v>
       </c>
     </row>
-    <row r="241" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A241" s="236">
         <v>2035</v>
       </c>
@@ -18708,7 +18761,7 @@
         <v>1084</v>
       </c>
     </row>
-    <row r="242" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242" s="236">
         <v>2035</v>
       </c>
@@ -18773,7 +18826,7 @@
         <v>1085</v>
       </c>
     </row>
-    <row r="243" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A243" s="236">
         <v>2035</v>
       </c>
@@ -18838,7 +18891,7 @@
         <v>1086</v>
       </c>
     </row>
-    <row r="244" spans="1:25" s="242" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:26" s="242" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244" s="242">
         <v>2035</v>
       </c>
@@ -18903,7 +18956,7 @@
         <v>1054</v>
       </c>
     </row>
-    <row r="245" spans="1:25" s="248" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:26" s="248" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A245" s="248">
         <v>2035</v>
       </c>
@@ -18968,7 +19021,7 @@
         <v>1076</v>
       </c>
     </row>
-    <row r="246" spans="1:25" s="248" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:26" s="248" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A246" s="248">
         <v>2035</v>
       </c>
@@ -19030,7 +19083,7 @@
         <v>1123</v>
       </c>
     </row>
-    <row r="247" spans="1:25" s="103" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:26" s="103" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A247" s="103">
         <v>2040</v>
       </c>
@@ -19054,7 +19107,7 @@
       <c r="W247" s="106"/>
       <c r="X247" s="106"/>
     </row>
-    <row r="248" spans="1:25" s="113" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:26" s="113" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A248" s="113">
         <v>2040</v>
       </c>
@@ -19078,7 +19131,7 @@
       <c r="W248" s="116"/>
       <c r="X248" s="116"/>
     </row>
-    <row r="249" spans="1:25" s="176" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:26" s="176" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A249" s="176">
         <v>2040</v>
       </c>
@@ -19142,8 +19195,11 @@
       <c r="Y249" s="176" t="s">
         <v>915</v>
       </c>
-    </row>
-    <row r="250" spans="1:25" s="77" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="Z249" s="176" t="s">
+        <v>915</v>
+      </c>
+    </row>
+    <row r="250" spans="1:26" s="77" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250" s="77">
         <v>2050</v>
       </c>
@@ -19205,7 +19261,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="251" spans="1:25" s="23" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:26" s="23" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251" s="23">
         <v>2050</v>
       </c>
@@ -19267,7 +19323,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="252" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:26" s="51" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A252" s="51">
         <v>2050</v>
       </c>
@@ -19323,7 +19379,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="253" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:26" s="51" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A253" s="51">
         <v>2050</v>
       </c>
@@ -19379,7 +19435,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="254" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:26" s="51" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254" s="51">
         <v>2050</v>
       </c>
@@ -19435,7 +19491,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="255" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:26" s="51" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A255" s="51">
         <v>2050</v>
       </c>
@@ -19494,7 +19550,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="256" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:26" s="51" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A256" s="51">
         <v>2050</v>
       </c>
@@ -19553,7 +19609,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="257" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:26" s="51" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257" s="51">
         <v>2050</v>
       </c>
@@ -19612,7 +19668,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="258" spans="1:25" s="51" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:26" s="51" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A258" s="51">
         <v>2050</v>
       </c>
@@ -19674,7 +19730,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="259" spans="1:25" s="86" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:26" s="86" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259" s="87">
         <v>2050</v>
       </c>
@@ -19737,7 +19793,7 @@
       </c>
       <c r="Y259" s="87"/>
     </row>
-    <row r="260" spans="1:25" s="86" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:26" s="86" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260" s="87">
         <v>2050</v>
       </c>
@@ -19802,7 +19858,7 @@
       </c>
       <c r="Y260" s="87"/>
     </row>
-    <row r="261" spans="1:25" s="138" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:26" s="138" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A261" s="134">
         <v>2050</v>
       </c>
@@ -19863,7 +19919,7 @@
       </c>
       <c r="Y261" s="134"/>
     </row>
-    <row r="262" spans="1:25" s="138" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:26" s="138" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262" s="134">
         <v>2050</v>
       </c>
@@ -19926,7 +19982,7 @@
       </c>
       <c r="Y262" s="134"/>
     </row>
-    <row r="263" spans="1:25" s="138" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:26" s="138" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A263" s="134">
         <v>2050</v>
       </c>
@@ -19988,7 +20044,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="264" spans="1:25" s="138" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:26" s="138" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A264" s="134">
         <v>2050</v>
       </c>
@@ -20050,7 +20106,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="265" spans="1:25" s="138" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:26" s="138" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A265" s="134">
         <v>2050</v>
       </c>
@@ -20112,7 +20168,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="266" spans="1:25" s="138" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:26" s="138" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A266" s="134">
         <v>2050</v>
       </c>
@@ -20174,7 +20230,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="267" spans="1:25" s="138" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:26" s="138" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A267" s="134">
         <v>2050</v>
       </c>
@@ -20240,8 +20296,11 @@
       <c r="Y267" s="134" t="s">
         <v>700</v>
       </c>
-    </row>
-    <row r="268" spans="1:25" s="66" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="Z267" s="134" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="268" spans="1:26" s="66" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A268" s="66">
         <v>2050</v>
       </c>
@@ -20297,7 +20356,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="269" spans="1:25" s="66" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:26" s="66" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A269" s="66">
         <v>2050</v>
       </c>
@@ -20353,7 +20412,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="270" spans="1:25" s="66" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:26" s="66" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A270" s="66">
         <v>2050</v>
       </c>
@@ -20409,7 +20468,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="271" spans="1:25" s="66" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:26" s="66" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A271" s="66">
         <v>2050</v>
       </c>
@@ -20468,7 +20527,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="272" spans="1:25" s="66" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:26" s="66" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A272" s="66">
         <v>2050</v>
       </c>
@@ -20527,7 +20586,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="273" spans="1:25" s="66" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:26" s="66" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A273" s="66">
         <v>2050</v>
       </c>
@@ -20586,7 +20645,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="274" spans="1:25" s="66" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:26" s="66" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274" s="66">
         <v>2050</v>
       </c>
@@ -20645,7 +20704,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="275" spans="1:25" s="66" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:26" s="66" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A275" s="66">
         <v>2050</v>
       </c>
@@ -20704,7 +20763,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="276" spans="1:25" s="66" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:26" s="66" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A276" s="66">
         <v>2050</v>
       </c>
@@ -20768,8 +20827,11 @@
       <c r="Y276" s="66" t="s">
         <v>673</v>
       </c>
-    </row>
-    <row r="277" spans="1:25" s="66" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="Z276" s="66" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="277" spans="1:26" s="66" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A277" s="66">
         <v>2050</v>
       </c>
@@ -20825,7 +20887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="1:25" s="66" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:26" s="66" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A278" s="66">
         <v>2050</v>
       </c>
@@ -20881,7 +20943,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="279" spans="1:25" s="66" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:26" s="66" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A279" s="66">
         <v>2050</v>
       </c>
@@ -20937,7 +20999,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="280" spans="1:25" s="134" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:26" s="134" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A280" s="134">
         <v>2050</v>
       </c>
@@ -20993,7 +21055,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="281" spans="1:25" s="134" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:26" s="134" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A281" s="134">
         <v>2050</v>
       </c>
@@ -21049,7 +21111,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="282" spans="1:25" s="138" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:26" s="138" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A282" s="134">
         <v>2050</v>
       </c>
@@ -21112,7 +21174,7 @@
       </c>
       <c r="Y282" s="134"/>
     </row>
-    <row r="283" spans="1:25" s="138" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:26" s="138" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A283" s="134">
         <v>2050</v>
       </c>
@@ -21175,7 +21237,7 @@
       </c>
       <c r="Y283" s="134"/>
     </row>
-    <row r="284" spans="1:25" s="138" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:26" s="138" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A284" s="134">
         <v>2050</v>
       </c>
@@ -21238,7 +21300,7 @@
       </c>
       <c r="Y284" s="134"/>
     </row>
-    <row r="285" spans="1:25" s="138" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:26" s="138" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A285" s="134">
         <v>2050</v>
       </c>
@@ -21301,7 +21363,7 @@
       </c>
       <c r="Y285" s="134"/>
     </row>
-    <row r="286" spans="1:25" s="138" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:26" s="138" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A286" s="134">
         <v>2050</v>
       </c>
@@ -21364,7 +21426,7 @@
       </c>
       <c r="Y286" s="134"/>
     </row>
-    <row r="287" spans="1:25" s="138" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:26" s="138" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A287" s="134">
         <v>2050</v>
       </c>
@@ -21427,7 +21489,7 @@
       </c>
       <c r="Y287" s="134"/>
     </row>
-    <row r="288" spans="1:25" s="138" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:26" s="138" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A288" s="134">
         <v>2050</v>
       </c>
@@ -21492,7 +21554,7 @@
       </c>
       <c r="Y288" s="134"/>
     </row>
-    <row r="289" spans="1:25" s="138" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:26" s="138" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A289" s="134">
         <v>2050</v>
       </c>
@@ -21560,8 +21622,11 @@
       <c r="Y289" s="134" t="s">
         <v>699</v>
       </c>
-    </row>
-    <row r="290" spans="1:25" s="173" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="Z289" s="134" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="290" spans="1:26" s="173" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A290" s="168">
         <v>2050</v>
       </c>
@@ -21626,7 +21691,7 @@
       </c>
       <c r="Y290" s="168"/>
     </row>
-    <row r="291" spans="1:25" s="173" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:26" s="173" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A291" s="168">
         <v>2050</v>
       </c>
@@ -21694,8 +21759,11 @@
       <c r="Y291" s="168" t="s">
         <v>876</v>
       </c>
-    </row>
-    <row r="292" spans="1:25" s="161" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="Z291" s="168" t="s">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="292" spans="1:26" s="161" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A292" s="156">
         <v>2050</v>
       </c>
@@ -21763,8 +21831,11 @@
       <c r="Y292" s="156" t="s">
         <v>902</v>
       </c>
-    </row>
-    <row r="293" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="Z292" s="156" t="s">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="293" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A293" s="236">
         <v>2050</v>
       </c>
@@ -21829,7 +21900,7 @@
         <v>1066</v>
       </c>
     </row>
-    <row r="294" spans="1:25" s="236" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:26" s="236" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A294" s="236">
         <v>2050</v>
       </c>
@@ -21894,7 +21965,7 @@
         <v>1067</v>
       </c>
     </row>
-    <row r="295" spans="1:25" s="254" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:26" s="254" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A295" s="236">
         <v>2050</v>
       </c>
@@ -21963,7 +22034,7 @@
         <v>1068</v>
       </c>
     </row>
-    <row r="296" spans="1:25" s="254" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:26" s="254" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A296" s="236">
         <v>2050</v>
       </c>
@@ -22032,7 +22103,7 @@
         <v>1069</v>
       </c>
     </row>
-    <row r="297" spans="1:25" s="254" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:26" s="254" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A297" s="236">
         <v>2050</v>
       </c>
@@ -22101,7 +22172,7 @@
         <v>1070</v>
       </c>
     </row>
-    <row r="298" spans="1:25" s="254" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:26" s="254" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A298" s="254">
         <v>2050</v>
       </c>
@@ -22164,6 +22235,19 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:Z298" xr:uid="{9564CC59-3725-4FDA-8BF2-0F68CB1B6F5A}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="RTP2025"/>
+        <filter val="RTP2025_IP"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="8">
+      <filters>
+        <filter val="current"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="M10" r:id="rId1" xr:uid="{1BE7DD4C-B567-4320-9B69-E8B55CE41797}"/>

</xml_diff>